<commit_message>
CAIQ round 2: 60.8% -> 64.2%, honest math on why 80% needs the pentest
Updated the completed xlsx and assessment doc with the round-2 answers
(15 more questions changed, backed by the interoperability policy,
governance addendum, and the annual-review-cadence additions).

Added an explicit "is 80% reachable" section: no, not through more
documentation or infrastructure work alone. Three domains are
structurally capped by things that take calendar time rather than
engineering effort -- TVM needs an independent pentest, Audit &
Assurance needs an independent assessment (literally requires
"independent" per 3 of its 8 questions), HR needs real hiring growth.
Multi-AZ infrastructure would add an estimated +5-6 points (~69-70%),
not enough alone to reach 80%. The pentest is the single highest-
leverage remaining lever.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ADMA_CAIQ_v4.0.3_Completed_2026-08-05.xlsx
+++ b/ADMA_CAIQ_v4.0.3_Completed_2026-08-05.xlsx
@@ -1028,9 +1028,9 @@
           <t xml:space="preserve">Are the policies and procedures reviewed and updated at least annually?</t>
         </is>
       </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The app runs on a single EC2 instance with no documented BCP/DR plan, no failover/redundancy, and no tested recovery procedure. UPDATE 2026-08-05: no explicit annual-review commitment yet for the DR plan specifically, though RISK_REGISTER.md's quarterly cadence touches the underlying risk.</t>
+          <t xml:space="preserve">The app runs on a single EC2 instance with no documented BCP/DR plan, no failover/redundancy, and no tested recovery procedure. UPDATE 2026-08-05: no explicit annual-review commitment yet for the DR plan specifically, though RISK_REGISTER.md's quarterly cadence touches the underlying risk. UPDATE 2026-08-05 (round 2): DISASTER_RECOVERY_PLAN.md now explicitly commits to annual review (Section 6).</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1280,9 +1280,9 @@
           <t xml:space="preserve">Is business continuity and operational resilience documentation reviewed periodically?</t>
         </is>
       </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The app runs on a single EC2 instance with no documented BCP/DR plan, no failover/redundancy, and no tested recovery procedure. UPDATE 2026-08-05: no explicit periodic-review commitment yet for the DR docs specifically.</t>
+          <t xml:space="preserve">The app runs on a single EC2 instance with no documented BCP/DR plan, no failover/redundancy, and no tested recovery procedure. UPDATE 2026-08-05: no explicit periodic-review commitment yet for the DR docs specifically. UPDATE 2026-08-05 (round 2): same DR plan review-cadence commitment covers this documentation.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1574,9 +1574,9 @@
           <t xml:space="preserve">Is the disaster response plan updated at least annually, and when significant changes occur?</t>
         </is>
       </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1586,7 +1586,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The app runs on a single EC2 instance with no documented BCP/DR plan, no failover/redundancy, and no tested recovery procedure. UPDATE 2026-08-05: no explicit annual-review commitment yet.</t>
+          <t xml:space="preserve">The app runs on a single EC2 instance with no documented BCP/DR plan, no failover/redundancy, and no tested recovery procedure. UPDATE 2026-08-05: no explicit annual-review commitment yet. UPDATE 2026-08-05 (round 2): same DR plan review-cadence commitment covers the disaster response plan specifically.</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1784,9 +1784,9 @@
           <t xml:space="preserve">Are the policies and procedures reviewed and updated at least annually?</t>
         </is>
       </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -1796,7 +1796,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Changes are tracked in git and deployed via a manual `git pull` + `pm2 restart` process on the EC2 host; there is no CI/CD pipeline, automated test gate, or formal Change Advisory process.</t>
+          <t xml:space="preserve">Changes are tracked in git and deployed via a manual `git pull` + `pm2 restart` process on the EC2 host; there is no CI/CD pipeline, automated test gate, or formal Change Advisory process. UPDATE 2026-08-05 (round 2): CHANGE_MANAGEMENT.md now explicitly commits to annual review (Section 6).</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -2246,9 +2246,9 @@
           <t xml:space="preserve">Are cryptography, encryption, and key management policies and procedures reviewed and updated at least annually?</t>
         </is>
       </c>
-      <c r="C51" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No formal key management policy, rotation schedule, or HSM/KMS customer-managed key usage — relies on AWS-managed default keys. UPDATE 2026-08-05: no explicit annual-review commitment stated yet in the new policy doc.</t>
+          <t xml:space="preserve">No formal key management policy, rotation schedule, or HSM/KMS customer-managed key usage — relies on AWS-managed default keys. UPDATE 2026-08-05: no explicit annual-review commitment stated yet in the new policy doc. UPDATE 2026-08-05 (round 2): KEY_MANAGEMENT_POLICY.md now explicitly commits to annual review (Section 5).</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -4178,9 +4178,9 @@
           <t xml:space="preserve">Are data security and privacy policies and procedures reviewed and updated at least annually?</t>
         </is>
       </c>
-      <c r="C97" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Server-side ownership scoping limits data access to the correct user/exhibitor, and sensitive fields (password_hash, totp_secret) are stripped from API responses, but there is no formal data classification scheme, documented retention/deletion schedule, or automated data-subject request workflow.</t>
+          <t xml:space="preserve">Server-side ownership scoping limits data access to the correct user/exhibitor, and sensitive fields (password_hash, totp_secret) are stripped from API responses, but there is no formal data classification scheme, documented retention/deletion schedule, or automated data-subject request workflow. UPDATE 2026-08-05 (round 2): DATA_CLASSIFICATION_AND_RETENTION.md now explicitly commits to annual review (Section 5).</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -5312,9 +5312,9 @@
           <t xml:space="preserve">Is an approved exception process mandated by the governance program established and followed whenever a deviation from an established policy occurs?</t>
         </is>
       </c>
-      <c r="C124" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C124" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
@@ -5324,7 +5324,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No formal risk register, InfoSec governance body, or documented risk assessment methodology exists.</t>
+          <t xml:space="preserve">No formal risk register, InfoSec governance body, or documented risk assessment methodology exists. UPDATE 2026-08-05 (round 2): GOVERNANCE_ADDENDUM.md Section 1 establishes a real, if lightweight, policy exception process.</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -5690,9 +5690,9 @@
           <t xml:space="preserve">Are the policies and procedures for defining allowances and conditions for the acceptable use of organizationally-owned or managed assets reviewed and updated at least annually?</t>
         </is>
       </c>
-      <c r="C133" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
@@ -5702,7 +5702,7 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No documented acceptable-use policy or signed confidentiality/NDA agreements on file. UPDATE 2026-08-05: no explicit annual-review commitment stated in the AUP yet.</t>
+          <t xml:space="preserve">No documented acceptable-use policy or signed confidentiality/NDA agreements on file. UPDATE 2026-08-05: no explicit annual-review commitment stated in the AUP yet. UPDATE 2026-08-05 (round 2): ACCEPTABLE_USE_POLICY.md now explicitly commits to annual review (Section 5).</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -7244,9 +7244,9 @@
           <t xml:space="preserve">Are policies and procedures established, documented, approved, communicated, applied, evaluated, and maintained for communications between application services (e.g., APIs)?</t>
         </is>
       </c>
-      <c r="C170" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C170" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -7256,7 +7256,7 @@
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No formal API versioning policy, published API documentation, or data portability/export guarantee is documented.</t>
+          <t xml:space="preserve">No formal API versioning policy, published API documentation, or data portability/export guarantee is documented. UPDATE 2026-08-05 (round 2): security/INTEROPERABILITY_AND_API_POLICY.md Section 1 documents the API communication standard.</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
@@ -7286,9 +7286,9 @@
           <t xml:space="preserve">Are policies and procedures established, documented, approved, communicated, applied, evaluated, and maintained for information processing interoperability?</t>
         </is>
       </c>
-      <c r="C171" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C171" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -7298,7 +7298,7 @@
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No formal API versioning policy, published API documentation, or data portability/export guarantee is documented.</t>
+          <t xml:space="preserve">No formal API versioning policy, published API documentation, or data portability/export guarantee is documented. UPDATE 2026-08-05 (round 2): same policy doc Section 3 documents information-processing interoperability.</t>
         </is>
       </c>
       <c r="F171" s="2" t="inlineStr">
@@ -7328,9 +7328,9 @@
           <t xml:space="preserve">Are policies and procedures established, documented, approved, communicated, applied, evaluated, and maintained for application development portability?</t>
         </is>
       </c>
-      <c r="C172" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C172" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -7340,7 +7340,7 @@
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No formal API versioning policy, published API documentation, or data portability/export guarantee is documented.</t>
+          <t xml:space="preserve">No formal API versioning policy, published API documentation, or data portability/export guarantee is documented. UPDATE 2026-08-05 (round 2): same policy doc Section 2 documents application development portability.</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
@@ -7412,9 +7412,9 @@
           <t xml:space="preserve">Are interoperability and portability policies and procedures reviewed and updated at least annually?</t>
         </is>
       </c>
-      <c r="C174" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No formal API versioning policy, published API documentation, or data portability/export guarantee is documented.</t>
+          <t xml:space="preserve">No formal API versioning policy, published API documentation, or data portability/export guarantee is documented. UPDATE 2026-08-05 (round 2): the new policy doc explicitly commits to annual review (Section 5).</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
@@ -9176,9 +9176,9 @@
           <t xml:space="preserve">Are information security incident metrics established and monitored?</t>
         </is>
       </c>
-      <c r="C216" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C216" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -9188,7 +9188,7 @@
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No documented incident response plan or breach notification procedure exists; the one real incident to date (a 2026-07-26 CSP rollout regression) was handled reactively rather than through a formal IR process.</t>
+          <t xml:space="preserve">No documented incident response plan or breach notification procedure exists; the one real incident to date (a 2026-07-26 CSP rollout regression) was handled reactively rather than through a formal IR process. UPDATE 2026-08-05 (round 2): GOVERNANCE_ADDENDUM.md Section 3 defines concrete incident metrics (severity counts, MTTC, MTTR, CSP violations, failed-login events), now queryable via centralized CloudWatch Logs.</t>
         </is>
       </c>
       <c r="F216" s="2" t="inlineStr">
@@ -9344,9 +9344,9 @@
           <t xml:space="preserve">Are points of contact maintained for applicable regulation authorities, national and local law enforcement, and other legal jurisdictional authorities?</t>
         </is>
       </c>
-      <c r="C220" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C220" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -9356,7 +9356,7 @@
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No documented incident response plan or breach notification procedure exists; the one real incident to date (a 2026-07-26 CSP rollout regression) was handled reactively rather than through a formal IR process.</t>
+          <t xml:space="preserve">No documented incident response plan or breach notification procedure exists; the one real incident to date (a 2026-07-26 CSP rollout regression) was handled reactively rather than through a formal IR process. UPDATE 2026-08-05 (round 2): GOVERNANCE_ADDENDUM.md Section 4 establishes an internal routing process for law-enforcement/regulatory requests, though no specific named external contact has been established yet.</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
@@ -9764,9 +9764,9 @@
           <t xml:space="preserve">Do service agreements between CSPs and CSCs (tenants) incorporate at least the following mutually agreed upon provisions and/or terms? • Scope, characteristics, and location of business relationship and services offered • Information security requirements (including SSRM) • Change management process • Logging and monitoring capability • Incident management and communication procedures • Right to audit and third-party assessment • Service termination • Interoperability and portability requirements • Data privacy</t>
         </is>
       </c>
-      <c r="C230" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C230" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partial</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -9776,7 +9776,7 @@
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No formal supplier/vendor security risk assessment process; dependencies are chosen for reputation/fit, not through a documented review.</t>
+          <t xml:space="preserve">No formal supplier/vendor security risk assessment process; dependencies are chosen for reputation/fit, not through a documented review. UPDATE 2026-08-05 (round 2): GOVERNANCE_ADDENDUM.md Section 5 acknowledges the gap and commits to a bundled legal review; VENDOR_DEPENDENCY_REVIEW.md already documents most of the substance informally.</t>
         </is>
       </c>
       <c r="F230" s="2" t="inlineStr">

</xml_diff>

<commit_message>
CAIQ round 3: 64.2% -> 64.8%, and update the public security report
Warm-standby infrastructure directly and cleanly answers BCR-11.1
("redundant equipment independently located") -- a correctly-honest
"No" through rounds 1-2 since no such redundancy existed yet. Business
Continuity Management moved 69.4% -> 77.8%.

Updated public/security-report.html (the ELI5 briefing, live at
admadigital.co.zw/security-report.html) to match: score 64% -> 65%,
and moved "running on two servers" from the growing/in-progress list
to the done list, since it's genuinely live now.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ADMA_CAIQ_v4.0.3_Completed_2026-08-05.xlsx
+++ b/ADMA_CAIQ_v4.0.3_Completed_2026-08-05.xlsx
@@ -1112,9 +1112,9 @@
           <t xml:space="preserve">Are strategies developed to reduce the impact of, withstand, and recover from business disruptions in accordance with risk appetite?</t>
         </is>
       </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Partial</t>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The app runs on a single EC2 instance with no documented BCP/DR plan, no failover/redundancy, and no tested recovery procedure. UPDATE 2026-08-05: PITR, DLM automated snapshots, and EC2 auto-recovery are real, implemented strategies to withstand/recover from disruption.</t>
+          <t xml:space="preserve">The app runs on a single EC2 instance with no documented BCP/DR plan, no failover/redundancy, and no tested recovery procedure. UPDATE 2026-08-05: PITR, DLM automated snapshots, and EC2 auto-recovery are real, implemented strategies to withstand/recover from disruption. UPDATE 2026-08-06 (round 3): PITR, DLM automated snapshots, EC2 auto-recovery, and now a live warm-standby instance together are real, implemented strategies to withstand and recover from disruption -- not just documented intent.</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1700,9 +1700,9 @@
           <t xml:space="preserve">Is business-critical equipment supplemented with redundant equipment independently located at a reasonable minimum distance in accordance with applicable industry standards?</t>
         </is>
       </c>
-      <c r="C38" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No</t>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No documented DR/BCP plan; the app runs on a single EC2 instance with no failover — an instance or AZ failure would cause an outage with no automatic recovery path.</t>
+          <t xml:space="preserve">No documented DR/BCP plan; the app runs on a single EC2 instance with no failover — an instance or AZ failure would cause an outage with no automatic recovery path. UPDATE 2026-08-06 (round 3): a warm-standby EC2 instance is live in a different availability zone (af-south-1b vs the primary's af-south-1a) -- genuine redundant equipment, independently located per AWS's own AZ isolation design (separate power/network/facility). See security/PROMOTION_RUNBOOK.md.</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">

</xml_diff>